<commit_message>
Sustituye Jardín Encantado por Saltapins/Embalse de l'Alcora en el plan de Castellón
Actualiza planes-en-familia-castellon.html y el plan aplicado (JSON/Excel)
con el intercambio de lugares, y añade la foto del Embalse de l'Alcora
aportada por el usuario (sustituye la foto genérica de Pexels usada
anteriormente).
</commit_message>
<xml_diff>
--- a/tools/output/planes-familia/castellon/plan.xlsx
+++ b/tools/output/planes-familia/castellon/plan.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.castello.es/es/planetario1</t>
+          <t>https://www.castello.es/es/planetario-informacion-general</t>
         </is>
       </c>
       <c r="F2" s="2" t="b">
@@ -728,7 +728,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://viasverdes.com/en/itineraries/mar/index.asp</t>
+          <t>https://viasverdes.com/itinerarios/itinerario.asp?id=45</t>
         </is>
       </c>
       <c r="F7" s="2" t="b">
@@ -850,17 +850,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Jardín Encantado (Oropesa del Mar)</t>
+          <t>Saltapins (Morella)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Un parque temático dentro del complejo Magic World Resort, en Oropesa del Mar, con árboles que hablan, hadas y espectáculos con actores entre miles de flores de más de 50 especies distintas. Está pensado como una experiencia fantástica para los más pequeños, con pasacalles y personajes que interactúan con el público. Un plan de tarde diferente, entre naturaleza cuidada y teatro familiar.</t>
+          <t>Un circuito de aventura entre árboles junto al río Bergantes, cerca de Morella, con tirolinas, puentes tibetanos y lianas repartidos en varios recorridos según edad. Está pensado para que niños a partir de 6 años completen los circuitos con cierta autonomía mientras la familia observa desde abajo. Un buen complemento de aventura a una visita a Morella.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.magicworldresort.com/en/parks/jardin-encantado</t>
+          <t>https://www.saltapins.com/</t>
         </is>
       </c>
       <c r="F10" s="2" t="b">
@@ -868,18 +868,18 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Marina d'Or, 12594 Oropesa del Mar (Castellón)</t>
+          <t>Fàbrica Giner, paraje junto al río Bergantes, 12300 Morella (Castellón)</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Tus Casas Rurales (tuscasasrurales.com); Ruralzoom (ruralzoom.com); Zonaviajero (zonaviajero.com)</t>
+          <t>Tus Casas Rurales (tuscasasrurales.com); Zonaviajero (zonaviajero.com)</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,11 @@
       <c r="F11" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>A unos 50 km de la costa de Castellón</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="n">
         <v>3</v>
       </c>
@@ -978,17 +982,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>MIAU - Museo Inacabado de Arte Urbano (Fanzara)</t>
+          <t>Embalse de l'Alcora (Circuito Multiaventura)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Un pequeño pueblo del interior de Castellón cuyas fachadas se han convertido en un museo al aire libre, con más de 150 murales de artistas de todo el mundo. Pasear por sus calles es como recorrer una galería urbana a cielo abierto, sin horarios ni entrada. Un plan diferente para familias que quieran combinar arte y pueblo tranquilo, alejado de la costa.</t>
+          <t>Un circuito de aventura en plena naturaleza, junto al embalse de l'Alcora, con actividades como tirolina, puente tibetano, kayak y tiro con arco. Está pensado para todo tipo de público, familias incluidas, en un entorno de montaña muy distinto a la costa. Un plan con más adrenalina para las familias que buscan actividad física al aire libre.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://miau32.wixsite.com/miaufanzara</t>
+          <t>https://www.comunitatvalenciana.com/es/mediterraneo-en-accion/embalse-de-l-alcora</t>
         </is>
       </c>
       <c r="F13" s="2" t="b">
@@ -996,18 +1000,18 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Plaça de l'Església, s/n, 12222 Fanzara (Castellón)</t>
+          <t>Paratge la Foia, Embassament de l'Alcora, 12110 l'Alcora (Castellón)</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Familias en Ruta (familiasenruta.com); Tus Casas Rurales (tuscasasrurales.com); Ruralzoom (ruralzoom.com)</t>
+          <t>Comunitat Valenciana (comunitatvalenciana.com); El Periódic (elperiodic.com)</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1080,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://parquesnaturales.gva.es/va/web/pn-serra-d-espada</t>
+          <t>https://parquesnaturales.gva.es/es/web/pn-serra-d-espada</t>
         </is>
       </c>
       <c r="F15" s="2" t="b">
@@ -1198,32 +1202,36 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Embalse de l'Alcora (Circuito Multiaventura)</t>
+          <t>Jardín Encantado (Oropesa del Mar)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Un circuito de aventura en plena naturaleza, junto al embalse de l'Alcora, con actividades como tirolina, puente tibetano, kayak y tiro con arco. Está pensado para todo tipo de público, familias incluidas, en un entorno de montaña muy distinto a la costa. Un plan con más adrenalina para las familias que buscan actividad física al aire libre.</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+          <t>Un parque temático dentro del complejo Magic World Resort, en Oropesa del Mar, con árboles que hablan, hadas y espectáculos con actores entre miles de flores de más de 50 especies distintas. Está pensado como una experiencia fantástica para los más pequeños, con pasacalles y personajes que interactúan con el público. Un plan de tarde diferente, entre naturaleza cuidada y teatro familiar.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.magicworldresort.com/es/parques/jardin-encantado</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Paratge la Foia, Embassament de l'Alcora, 12110 l'Alcora (Castellón)</t>
+          <t>Marina d'Or, 12594 Oropesa del Mar (Castellón)</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Comunitat Valenciana (comunitatvalenciana.com); El Periódic (elperiodic.com)</t>
+          <t>Tus Casas Rurales (tuscasasrurales.com); Ruralzoom (ruralzoom.com); Zonaviajero (zonaviajero.com)</t>
         </is>
       </c>
     </row>
@@ -1238,17 +1246,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Saltapins (Morella)</t>
+          <t>MIAU - Museo Inacabado de Arte Urbano (Fanzara)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Un circuito de aventura entre árboles junto al río Bergantes, cerca de Morella, con tirolinas, puentes tibetanos y lianas repartidos en varios recorridos según edad. Está pensado para que niños a partir de 6 años completen los circuitos con cierta autonomía mientras la familia observa desde abajo. Un buen complemento de aventura a una visita a Morella.</t>
+          <t>Un pequeño pueblo del interior de Castellón cuyas fachadas se han convertido en un museo al aire libre, con más de 150 murales de artistas de todo el mundo. Pasear por sus calles es como recorrer una galería urbana a cielo abierto, sin horarios ni entrada. Un plan diferente para familias que quieran combinar arte y pueblo tranquilo, alejado de la costa.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.saltapins.com/</t>
+          <t>https://miau32.wixsite.com/miaufanzara-2016</t>
         </is>
       </c>
       <c r="F19" s="2" t="b">
@@ -1256,18 +1264,18 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Fàbrica Giner, paraje junto al río Bergantes, 12300 Morella (Castellón)</t>
+          <t>Plaça de l'Església, s/n, 12222 Fanzara (Castellón)</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Tus Casas Rurales (tuscasasrurales.com); Zonaviajero (zonaviajero.com)</t>
+          <t>Familias en Ruta (familiasenruta.com); Tus Casas Rurales (tuscasasrurales.com); Ruralzoom (ruralzoom.com)</t>
         </is>
       </c>
     </row>

</xml_diff>